<commit_message>
feat: add WMS logistics application modules including inventory management page, sales store, and UI components
</commit_message>
<xml_diff>
--- a/server/data/plantilla_despachos_vehiculos.xlsx
+++ b/server/data/plantilla_despachos_vehiculos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="17">
   <si>
     <t>Número de factura</t>
   </si>
@@ -28,7 +28,7 @@
     <t>FE-90001</t>
   </si>
   <si>
-    <t>2026-09-14 20:03:12</t>
+    <t>2026-09-14 20:57:16</t>
   </si>
   <si>
     <t>FE-90003</t>
@@ -40,10 +40,7 @@
     <t>FE-80297</t>
   </si>
   <si>
-    <t>2026-09-14T20:03:12.416Z</t>
-  </si>
-  <si>
-    <t>2026-09-14T20:31:30.976Z</t>
+    <t>2026-09-14T20:57:17.118Z</t>
   </si>
   <si>
     <t>FE-90002</t>
@@ -466,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -526,17 +523,6 @@
         <v>8</v>
       </c>
       <c r="C5" s="3">
-        <v>5840000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="3">
         <v>5840000</v>
       </c>
     </row>
@@ -569,7 +555,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -580,7 +566,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
@@ -618,7 +604,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -629,7 +615,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
@@ -640,7 +626,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
@@ -678,7 +664,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -689,7 +675,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
@@ -700,7 +686,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
feat: implement WMS dispatch management system with React context and OneDrive Excel integration
</commit_message>
<xml_diff>
--- a/server/data/plantilla_despachos_vehiculos.xlsx
+++ b/server/data/plantilla_despachos_vehiculos.xlsx
@@ -4,43 +4,88 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="WRO-482" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="STZ-910" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="ENV-301" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="MC-441" state="visible" r:id="rId7"/>
+    <sheet sheetId="1" name="WDO-069 ANDERSON" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="TJP-653 GRIS" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="A20BB5E JEFERSON" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="WDP-097 JESUS" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="17">
-  <si>
-    <t>Número de factura</t>
-  </si>
-  <si>
-    <t>Fecha</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="34">
+  <si>
+    <t>CONTROL DE DESPACHO A CLIENTES</t>
+  </si>
+  <si>
+    <t>Versión: 1</t>
+  </si>
+  <si>
+    <t>Fecha: 14/09/2026</t>
+  </si>
+  <si>
+    <t>Vehículo: WDO-069 ANDERSON</t>
+  </si>
+  <si>
+    <t>Nombre del cliente</t>
+  </si>
+  <si>
+    <t>Dirección</t>
+  </si>
+  <si>
+    <t>AM</t>
+  </si>
+  <si>
+    <t>PM</t>
+  </si>
+  <si>
+    <t>Número de Factura</t>
   </si>
   <si>
     <t>Valor de la factura</t>
   </si>
   <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Firma de Recibido</t>
+  </si>
+  <si>
+    <t>S/N</t>
+  </si>
+  <si>
+    <t>S/D</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>FE-90001</t>
   </si>
   <si>
-    <t>2026-09-14 20:57:16</t>
-  </si>
-  <si>
     <t>FE-90003</t>
   </si>
   <si>
     <t>FE-CONC-4</t>
   </si>
   <si>
+    <t>Ferretería La Campana S.A.S.</t>
+  </si>
+  <si>
+    <t>Av 5 # 10-45</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
     <t>FE-80297</t>
   </si>
   <si>
-    <t>2026-09-14T20:57:17.118Z</t>
+    <t>SUBTOTAL</t>
+  </si>
+  <si>
+    <t>Vehículo: TJP-653 GRIS</t>
   </si>
   <si>
     <t>FE-90002</t>
@@ -49,6 +94,9 @@
     <t>FE-CONC-6</t>
   </si>
   <si>
+    <t>Vehículo: A20BB5E JEFERSON</t>
+  </si>
+  <si>
     <t>FE-CONC-1</t>
   </si>
   <si>
@@ -56,6 +104,9 @@
   </si>
   <si>
     <t>FE-CONC-7</t>
+  </si>
+  <si>
+    <t>Vehículo: WDP-097 JESUS</t>
   </si>
   <si>
     <t>FE-CONC-3</t>
@@ -74,7 +125,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -84,8 +135,18 @@
     </font>
     <font>
       <b/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -113,9 +174,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -124,6 +192,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,70 +535,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="5" customWidth="1"/>
+    <col min="5" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3">
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6">
         <v>4500000</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="6">
         <v>7200000</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3">
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="6">
         <v>400000</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="3">
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="6">
         <v>5840000</v>
       </c>
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="8">
+        <v>17940000</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -534,48 +729,141 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="5" customWidth="1"/>
+    <col min="5" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="E5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3">
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="6">
         <v>1800000</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="6">
         <v>600000</v>
       </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="8">
+        <v>2400000</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -583,59 +871,167 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="5" customWidth="1"/>
+    <col min="5" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="E5" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="6">
         <v>100000</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="6">
         <v>200000</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3">
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="6">
         <v>700000</v>
       </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1000000</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -643,59 +1039,167 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="5" customWidth="1"/>
+    <col min="5" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3">
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="6">
         <v>300000</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="6">
         <v>500000</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3">
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="6">
         <v>800000</v>
       </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1600000</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement WmsContext with two-state dispatch model and OneDrive synchronization
</commit_message>
<xml_diff>
--- a/server/data/plantilla_despachos_vehiculos.xlsx
+++ b/server/data/plantilla_despachos_vehiculos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="38">
   <si>
     <t>CONTROL DE DESPACHO A CLIENTES</t>
   </si>
@@ -80,6 +80,18 @@
   </si>
   <si>
     <t>FE-80297</t>
+  </si>
+  <si>
+    <t>ferre largo</t>
+  </si>
+  <si>
+    <t>av 6 b</t>
+  </si>
+  <si>
+    <t>PR 0001</t>
+  </si>
+  <si>
+    <t>vvvv</t>
   </si>
   <si>
     <t>SUBTOTAL</t>
@@ -535,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -709,12 +721,38 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="8">
-        <v>17940000</v>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="6">
+        <v>110000</v>
+      </c>
+      <c r="G11" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="8">
+        <v>18050000</v>
       </c>
     </row>
   </sheetData>
@@ -770,7 +808,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -813,7 +851,7 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F7" s="6">
         <v>1800000</v>
@@ -839,7 +877,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F8" s="6">
         <v>600000</v>
@@ -853,7 +891,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F9" s="8">
         <v>2400000</v>
@@ -912,7 +950,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -955,7 +993,7 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F7" s="6">
         <v>100000</v>
@@ -981,7 +1019,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F8" s="6">
         <v>200000</v>
@@ -1007,7 +1045,7 @@
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F9" s="6">
         <v>700000</v>
@@ -1021,7 +1059,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F10" s="8">
         <v>1000000</v>
@@ -1080,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1123,7 +1161,7 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F7" s="6">
         <v>300000</v>
@@ -1149,7 +1187,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F8" s="6">
         <v>500000</v>
@@ -1175,7 +1213,7 @@
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F9" s="6">
         <v>800000</v>
@@ -1189,7 +1227,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F10" s="8">
         <v>1600000</v>

</xml_diff>

<commit_message>
feat: add WmsContext for dispatch state management and vehicle Excel template
</commit_message>
<xml_diff>
--- a/server/data/plantilla_despachos_vehiculos.xlsx
+++ b/server/data/plantilla_despachos_vehiculos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="46">
   <si>
     <t>CONTROL DE DESPACHO A CLIENTES</t>
   </si>
@@ -106,6 +106,18 @@
     <t>FE-CONC-6</t>
   </si>
   <si>
+    <t>ferre andre</t>
+  </si>
+  <si>
+    <t>av 5 6e</t>
+  </si>
+  <si>
+    <t>PR 002</t>
+  </si>
+  <si>
+    <t>jjsjsjsjs</t>
+  </si>
+  <si>
     <t>Vehículo: A20BB5E JEFERSON</t>
   </si>
   <si>
@@ -128,6 +140,18 @@
   </si>
   <si>
     <t>FE-CONC-8</t>
+  </si>
+  <si>
+    <t>ferre j</t>
+  </si>
+  <si>
+    <t>av 6 e casa 1</t>
+  </si>
+  <si>
+    <t>PR 003</t>
+  </si>
+  <si>
+    <t>kskksaksd</t>
   </si>
 </sst>
 </file>
@@ -581,8 +605,8 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>2</v>
@@ -767,7 +791,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -889,12 +913,38 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="6">
+        <v>100000</v>
+      </c>
+      <c r="G9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="8">
-        <v>2400000</v>
+      <c r="F10" s="8">
+        <v>2500000</v>
       </c>
     </row>
   </sheetData>
@@ -950,7 +1000,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -993,7 +1043,7 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F7" s="6">
         <v>100000</v>
@@ -1019,7 +1069,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F8" s="6">
         <v>200000</v>
@@ -1045,7 +1095,7 @@
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F9" s="6">
         <v>700000</v>
@@ -1077,7 +1127,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -1111,14 +1161,14 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1161,7 +1211,7 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F7" s="6">
         <v>300000</v>
@@ -1187,7 +1237,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F8" s="6">
         <v>500000</v>
@@ -1213,7 +1263,7 @@
         <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F9" s="6">
         <v>800000</v>
@@ -1225,12 +1275,38 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="6">
+        <v>100050</v>
+      </c>
+      <c r="G10" t="s">
+        <v>45</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="8">
-        <v>1600000</v>
+      <c r="F11" s="8">
+        <v>1700050</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement WMS dispatch module with UI components, backend controller, and Excel template synchronization
</commit_message>
<xml_diff>
--- a/server/data/plantilla_despachos_vehiculos.xlsx
+++ b/server/data/plantilla_despachos_vehiculos.xlsx
@@ -14,19 +14,121 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="35">
   <si>
     <t>CONTROL DE DESPACHO A CLIENTES</t>
   </si>
   <si>
     <t>Versión: 1</t>
+  </si>
+  <si>
+    <t>Fecha: 16/09/2026</t>
+  </si>
+  <si>
+    <t>Vehículo: WDO-069 ANDERSON</t>
+  </si>
+  <si>
+    <t>Nombre del cliente</t>
+  </si>
+  <si>
+    <t>Dirección</t>
+  </si>
+  <si>
+    <t>AM</t>
+  </si>
+  <si>
+    <t>PM</t>
+  </si>
+  <si>
+    <t>Número de Factura</t>
+  </si>
+  <si>
+    <t>Valor de la factura</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Firma de Recibido</t>
+  </si>
+  <si>
+    <t>S/N</t>
+  </si>
+  <si>
+    <t>S/D</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>FE-90001</t>
+  </si>
+  <si>
+    <t>FE-90003</t>
+  </si>
+  <si>
+    <t>FE-CONC-4</t>
+  </si>
+  <si>
+    <t>SUBTOTAL</t>
+  </si>
+  <si>
+    <t>Fecha: 15/09/2026</t>
+  </si>
+  <si>
+    <t>Ferretería La Campana S.A.S.</t>
+  </si>
+  <si>
+    <t>Av 5 # 10-45</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>FE-80297</t>
+  </si>
+  <si>
+    <t>Vehículo: TJP-653 GRIS</t>
+  </si>
+  <si>
+    <t>FE-90002</t>
+  </si>
+  <si>
+    <t>FE-CONC-6</t>
+  </si>
+  <si>
+    <t>Vehículo: A20BB5E JEFERSON</t>
+  </si>
+  <si>
+    <t>FE-CONC-1</t>
+  </si>
+  <si>
+    <t>FE-CONC-2</t>
+  </si>
+  <si>
+    <t>FE-CONC-7</t>
+  </si>
+  <si>
+    <t>Vehículo: WDP-097 JESUS</t>
+  </si>
+  <si>
+    <t>FE-CONC-3</t>
+  </si>
+  <si>
+    <t>FE-CONC-5</t>
+  </si>
+  <si>
+    <t>FE-CONC-8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -42,13 +144,25 @@
       <i/>
       <sz val="10"/>
     </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE11D24"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -63,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -71,6 +185,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -444,21 +572,209 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6">
+        <v>4500000</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="6">
+        <v>7200000</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="6">
+        <v>400000</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="8">
+        <v>12100000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="6">
+        <v>5840000</v>
+      </c>
+      <c r="G14" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="8">
+        <v>5840000</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -494,19 +810,113 @@
     </row>
     <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="6">
+        <v>1800000</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="6">
+        <v>600000</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="8">
+        <v>2400000</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -542,19 +952,139 @@
     </row>
     <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="6">
+        <v>100000</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="6">
+        <v>200000</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="6">
+        <v>700000</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1000000</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -590,12 +1120,132 @@
     </row>
     <row r="3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="6">
+        <v>300000</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="6">
+        <v>500000</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="6">
+        <v>800000</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1600000</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add logistics dispatch management system with vehicle tracking and Google Drive sync
</commit_message>
<xml_diff>
--- a/server/data/plantilla_despachos_vehiculos.xlsx
+++ b/server/data/plantilla_despachos_vehiculos.xlsx
@@ -8,13 +8,14 @@
     <sheet sheetId="2" name="TJP-653 GRIS" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="A20BB5E JEFERSON" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="WDP-097 JESUS" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="XYZ-999 PRUEBA" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="23">
   <si>
     <t>Control de Despacho a Clientes</t>
   </si>
@@ -77,6 +78,12 @@
   </si>
   <si>
     <t>Placa de Vehículo : WDP-097 JESUS</t>
+  </si>
+  <si>
+    <t>Fecha: 04/10/2026</t>
+  </si>
+  <si>
+    <t>Placa de Vehículo : XYZ-999 PRUEBA</t>
   </si>
 </sst>
 </file>
@@ -86,7 +93,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;[Red]-&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -110,6 +117,9 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="4">
@@ -157,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -174,6 +184,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -704,7 +715,7 @@
     <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -901,7 +912,7 @@
     <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1098,7 +1109,7 @@
     <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1295,6 +1306,97 @@
     <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="4" width="6" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>